<commit_message>
Daily status update (run 36678317948)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="348642" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="348649" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="349661" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="349722" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="350050" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Employees" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="348642" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="348649" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="349661" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="349722" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="350050" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -79,12 +79,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -708,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -739,6 +745,48 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>29-09-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>1. test www
+2. 1. test xxx</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>1. test work 1
+2. test work 2</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily status update (run 36679336239)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -672,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -700,6 +700,28 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Blockers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>29-09-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>1. Designed and created the required database tables and indexes for the Raise Ticket / Support Dashboard feature.
+2. Structured the database to support Support Member management, service categories, support tickets, ticket assignment, ticket status tracking, document update requests, and related audit information.
+3. Finalized the database structure based on the provided Support Dashboard Database Schema reference and prepared it for further implementation.</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily status update (run 36697576143)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -778,8 +778,10 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>1. test www
-2. 1. test xxx</t>
+          <t>1. Team Discussion regarding the Order Document Mapping &amp; Version Resolution
+2. Updated the doc &amp; shared the team with respective Flow we finalised in meeting
+3. Created initial DB Schema for the support dashboard &amp; explained the team
+4. Modification noted &amp; required for device document mapping tables considering the ticket source by which Device doc has been updated</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Daily status update (run 36697823530)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -801,8 +801,8 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>1. test work 1
-2. test work 2</t>
+          <t>1. Reviewed the backend implementation approach document for device document re-upload prepared by Thirumal.
+2. Recommended including all predefined document categories in the JSON structure, even if no documents have been uploaded under a particular category, to maintain consistency across all orders.</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Daily status update (run 36709800089)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -616,6 +616,27 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Blockers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>29-09-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>1. Password Reset Functionality – Worked on the implementation approach for password reset functionality for Client, Admin, and Tester user roles – Ongoing
+2. Password Reset Architecture Mapping – Mapped the required architecture and implementation flow for handling password reset securely across the respective user roles – Ongoing</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily status update (run 36709999538)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -635,6 +635,31 @@
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>1. Change Password Backend API – Implemented the Change Password functionality for authenticated Client, Admin, and Tester users – Completed
+2. Implemented password validation, including current password verification, new password policy validation, confirm-password matching, and password reuse prevention – Completed
+3. Implemented secure password updates using bcrypt – Completed
+4. Implemented session revocation using revoked_at after a successful password change – Completed
+5. Updated the authentication middleware to reject revoked sessions – Completed
+6. Implemented the security flow to ensure the old authentication token is rejected after a password change – Completed</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 36711819043)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -676,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -704,6 +704,28 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Blockers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>1. Completed the document upload functionality during Client Device Registration, including the required document handling workflow.
+2. Completed the frontend implementation of the Device Details page based on the new document upload architecture.
+3. Currently working on the Raise Ticket workflow within the Device Details module, including the required functionality and integration with the new architecture.</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily status update (run 36717395179)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -574,6 +574,28 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Blockers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>29-09-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Task - 2602:
+Had a meeting with the team to finalize the device document re-upload feature.
+Prepared a document on the discussions held about the workflow.</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily status update (run 36717717141)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -594,6 +594,28 @@
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Task - 2602:
+1. Implemented order-level device document handling by storing the latest available document references in the order_documents JSONB field during order placement.
+2. Updated device document retrieval for Desktop DB integration, including MinIO path mapping and handling document re-upload updates.</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 36718463360)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -832,6 +832,28 @@
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>1. Started working on the Raise Ticket / Support Dashboard feature implementation and defining the overall workflow.
+2. Working on the scalable implementation approach, including ticket creation, assignment, status tracking, support member management, and document update requests.
+3. Reviewing the architecture and database integration to ensure the feature is **maintainable, scalable, and suitable for future enhancements.</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 36857644285)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -632,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -704,6 +704,27 @@
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>01-10-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1. Completed functional, negative, and security validation for the Change Password functionality across Client, Admin, and Tester user roles – Completed &amp; Verified
+2. Validated incorrect current password, password mismatch, invalid password format, password reuse, old token rejection, old password rejection, and login with the new password – Completed &amp; Tested</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 36858545117)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -789,6 +789,27 @@
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>01-10-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>1. Currently working on the Raise Ticket workflow within the Device Details module, focusing on implementing the required functionality in alignment with the new architecture.
+2. Initiated backend development for the Raise Ticket workflow, including the implementation of the necessary APIs and supporting logic.</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 36860853900)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -616,6 +616,27 @@
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>01-10-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1. Worked on the Integration service to store the updated device documents during order placement.
+2. Started working on updating documents when uploaded on the device details page.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37312740949)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -847,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -917,6 +917,28 @@
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>05-10-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1. Started working on the Raise Ticket / Support Dashboard frontend implementation based on the provided reference layout.
+2. Working on integrating the Super Admin screens for Service Categories and Support Service Team, along with the Support Member dashboard and ticket management flow.
+3. Reviewing the frontend architecture and existing authentication/role mechanism to ensure the implementation remains scalable and compatible with the existing Web Portal, without introducing a separate login or authentication system.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37315181930)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -637,6 +637,27 @@
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>05-10-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1. Created a controller for fetching order details when a document is updated.
+2. Fetched the updated document and replaced it in the orders table.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37416192718)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -976,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1051,6 +1051,28 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>05-10-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1. Researched the Security Sandbox.  
+2. Started designing the initial layout and content based on the discussions and insights shared during the event talks by Sam Sir.
+3. Created a task for integrating the Support Dashboard with the Web Portal.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily status update (run 37419113751)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -783,7 +783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -854,6 +854,27 @@
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>05-10-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1. Currently working on the Raise Ticket workflow within the Device Details module, focusing on integrating the required functionality with the new architecture.
+2. Completed the backend development for the Raise Ticket workflow, including the required APIs, business logic, and supporting functionality.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily status update (run 37461679441)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -769,6 +769,27 @@
       <c r="D4" s="4" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>06-10-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1. Pushed the completed Change Password code changes to the Server – Completed
+2. Completed the Change Password implementation and security testing documentation – Completed</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>The code has been pushed to the Server. The Frontend implementation is pending and needs to be completed by @Kurni Thirumala.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily status update (run 37464370543)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -804,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -894,6 +894,28 @@
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>06-10-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1. Modified the ticket data persistence flow in the `support_tickets` and `device_document_mapping` tables to align with the updated architecture.
+2. Completed the end-to-end Raise Ticket workflow for Device Registration, covering the required frontend and backend functionality.
+3. Completed the backend development for the Raise Ticket workflow, including the required APIs, business logic, and supporting functionality.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37571307529)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -932,7 +932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1024,6 +1024,28 @@
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>06-10-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued working on the Raise Ticket / Support Dashboard frontend implementation based on the provided reference layout.
+2. Continued implementation of the Super Admin screens for Service Categories and Support Service Team, along with the Support Member dashboard and ticket management flow.
+3. Continued reviewing and refining the frontend architecture and existing authentication/role mechanism to ensure the implementation remains scalable and compatible with the existing Web Portal.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1040,7 +1062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1137,6 +1159,27 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>06-10-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1. Meeting with team to have a KT session to freshers for Git &amp; Project Management Tool
+2. Research on security sandbox</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily status update (run 37571385413)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1062,7 +1062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1180,6 +1180,28 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>07-10-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1. Reserach On security sandbox
+2. Meeting with aboli new team mate to have an overall picture of web portal for QA start
+3. Attend the KT session from team with freshers</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily status update (run 37619408057)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -790,6 +790,26 @@
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>The code has been pushed to the Server. The Frontend implementation is pending and needs to be completed by @Kurni Thirumala.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>07-10-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1. API to Upload Generated Report Files to MinIO – Reviewed the API implementation, storage path configuration, environment-specific handling, authentication, authorization, file validation, and MinIO integration – Ongoing</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily status update (run 37620261843)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -824,7 +824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -938,6 +938,27 @@
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>07-10-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1. Completed the Device Details page and deployed the latest changes to the development environment for further testing and validation.
+2. Conducted a presentation for freshers on the Project Management Tool, covering how to access the tool, navigate the relevant sections, view project activities, and update task status and other required details.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily status update (run 37625193881)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -973,7 +973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1087,6 +1087,28 @@
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>07-10-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued working on the Raise Ticket / Support Dashboard frontend implementation and created a separate login page for Support Service Members.
+2. Configured the Support Member login flow so that only users with the Support Service Member role can access it, preventing other roles from logging in through this page.
+3. Added alerts and role-based restrictions to the main Web Portal login, clarifying that Support Service Members must use their dedicated login, while Client, Admin, Super Admin, and Tester users can continue using the main login.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37625599480)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -658,6 +658,26 @@
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>06-10-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Working on preparing a presentation on Git &amp; GitLab.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37625835017)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,26 @@
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>07-10-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Presented a Presentation for new joiners on Git &amp; GitLab.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37772197295)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1165,7 +1165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1305,6 +1305,29 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>08-10-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>1. Created the BUG EPIC and QA testing task.
+2. Explained the bug reporting workflow to the QA team, including the process for raising, documenting, and sharing bugs.
+3. Attended the Freshers session conducted by Aboli.
+4. Followed up with the team to discuss task roadblocks and required resolutions.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily status update (run 37773557095)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -714,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -848,6 +848,27 @@
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>08-10-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>1. API to Upload Generated Report Files to MinIO – Continued the review of the API implementation, including authentication, authorization, file validation, MinIO integration, storage configuration, and security considerations – Ongoing
+2. PM2 Server Issues – Identified and fixed the PM2-related issues on the server and verified the application services are running correctly – Completed &amp; Verified</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37776361750)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -885,7 +885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1020,6 +1020,28 @@
       <c r="D6" s="4" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>08-10-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>1. Started implementing the Client Device Registration document upload workflow, with documents being stored directly in MinIO.
+2. Completed the Device Details page and deployed the latest changes to the development environment for further testing and validation.
+3. Identified and resolved bugs related to device document handling and completed testing in the development environment to ensure the workflow functions as expected.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily status update (run 37779960365)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -698,6 +698,29 @@
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>08-10-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Task - 2602 : 
+1. Implemented and debugged the Update Device Documents gRPC integration.
+2. Fixed the gRPC handler export/registration issue causing UNIMPLEMENTED errors.
+3. Reviewed and optimized device document retrieval and order document snapshot logic.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37781263291)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1079,7 +1079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1215,6 +1215,28 @@
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>08-10-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued working on the Raise Ticket / Support Dashboard frontend implementation and the Support Service Member login flow.
+2. Created a demo Support Service Member user to test and verify that the dedicated login functionality is working correctly with the required role-based access.
+3. Continued testing the login restrictions and ensuring that only Support Service Members can access the dedicated login, while other roles are restricted from accessing it.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37926346690)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -737,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -892,6 +892,26 @@
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>09-10-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>1. API to Upload Generated Report Files to MinIO – Completed the API review and started implementing the required functionality, including file validation, authentication, authorization, and MinIO integration – Implementation Ongoing</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37928905756)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -928,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1083,6 +1083,28 @@
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>09-10-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>1. Completed the Client Device Registration document upload functionality, enabling direct document storage in MinIO during the registration process.
+2. Completed end-to-end testing of the Client Device Registration document upload workflow in the development environment.
+3. Identified and resolved bugs related to device document handling and performed regression testing in the development environment to ensure the workflow functions as expected.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37931830031)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -721,6 +721,28 @@
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>09-10-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>1. Updated the ongoing order document retrieval logic to select only the most recent order with ASSIGNED or IN_PROGRESS test assignments.
+2. Refined transaction management, error handling, and database connection cleanup for reliable document updates.
+3. Researched on Test Reports to prepare a Reports Template.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 37935717467)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1143,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1301,6 +1301,28 @@
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>09-10-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>1. Prepared a PowerPoint presentation covering the end-to-end client onboarding and Functionality Sandbox workflow in the IoT Security Ecosystem &amp; Sandbox Web Portal.
+2. Documented the step-by-step process, including client login, Functionality Sandbox navigation, device selection/registration, test configuration, and test request submission.
+3. Covered the C-DAC Bangalore workflow, test execution and status tracking, and generated test report availability in the client dashboard.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38245779360)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -950,7 +950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1127,6 +1127,29 @@
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>12-10-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>1. Identified and resolved bugs related to device document handling and performed regression testing in the development environment to ensure the workflow functions correctly and reliably.
+2. Implemented document uploads directly from the Select Services page, eliminating the need to redirect users to the Device Details page.
+3. Implemented document update functionality on the Select Services page, following the same workflow as the Device Details page.
+4. Pushed the code to the development server and tested the document upload and update workflows on the Select Services page to verify that they function as expected.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38247000656)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -759,7 +759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -934,6 +934,27 @@
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>12-10-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>1. MinIO Security Gap Analysis – Researched and reviewed potential security gaps in MinIO object storage – Completed
+2. CDAC Hyderabad Hardware Requirements – Researched the hardware requirements for the CDAC Hyderabad project – Completed</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38252126395)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1187,7 +1187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1367,6 +1367,29 @@
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>12-10-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>1. Completed the frontend implementation of the Raise Ticket / Support Desk feature, including the Support Member Dashboard and ticket management workflow.
+2. Implemented the Super Admin screens for Service Categories and Support Service Team management, along with role-based access and the ticket status actions.
+3. Added the Support Member Desk link to the Web Portal footer to provide direct access to the dedicated Support Desk login page.
+4. Aligned the Support Desk UI and interactions with the provided reference layout while reusing the existing Web Portal authentication mechanism.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38394592356)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1171,6 +1171,28 @@
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>13-10-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>1. Completed testing the device document upload and update request workflows on the Select Services page to verify that they function as expected.
+2. Tested the new document upload and download service by creating the required buckets and verifying the document handling workflow.
+3. Identified and resolved notification-related bugs to ensure the notification functionality works correctly.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38400073240)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1209,7 +1209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1412,6 +1412,28 @@
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>13-10-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>1. Started evaluating SecureStore as a potential replacement for the existing MinIO object storage solution.
+2. Working on setting up and testing the storage-service and upload-api locally, including dependency installation, automated tests, environment configuration, and service initialization.
+3. Reviewing the REST API functionality for bucket creation, file upload/download, listing, deletion, authentication, and error handling, along with local file storage and audit logs.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38564271387)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1193,6 +1193,27 @@
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>14-10-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>1. Completed testing the new storage service for document uploads using Postman to verify that the API functions as expected.
+2. Started integrating the new storage service into the local application code to enable document uploads through the updated service.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38566944601)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1230,7 +1230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1455,6 +1455,28 @@
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>14-10-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>1. Started the backend implementation of the Raise Ticket / Support Desk feature, following the completed frontend integration.
+2. Working on backend APIs and database integration for ticket creation, ticket management, and support team assignment.
+3. Implementing role-based access and backend functionality for Service Categories, Support Service Team management, and ticket status updates.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38571669713)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,28 @@
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>13-10-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>1. Analyzed reporting requirements across Functionality Sandbox, Security Sandbox, Device Security Solution, and Network Security Solution.
+2. Identified common report sections, mandatory fields, and vertical-specific requirements.
+3. Defined the overall structure for a standardized testing report.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38571752560)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -765,6 +765,27 @@
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>14-10-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>1. Designed a standardized format for presenting test cases, execution status, expected results, and actual results.
+2. Defined a consistent mechanism for incorporating screenshots, logs, test evidence, and supporting references.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38729623998)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1014,7 +1014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1257,6 +1257,27 @@
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>15-10-2026</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>1. Started integrating the new storage service into the local application code to enable document uploads through the updated service.
+2. Completed the backend implementation for document uploads using the new storage service.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38733386951)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1294,7 +1294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1541,6 +1541,28 @@
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>15-10-2026</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued the backend implementation of the Raise Ticket / Support Desk feature, building on the completed frontend integration.
+2. Continued working on backend APIs and database integration for ticket creation, ticket management, and support team assignment.
+3. Continued implementing role-based access control and backend functionality for Service Categories, Support Service Team management, and ticket status updates.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38897503339)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1014,7 +1014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1278,6 +1278,26 @@
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>16-10-2026</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>1. Started integrating the new storage service into the local application code to enable document uploads through the updated service.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38899533763)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -786,6 +786,26 @@
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>15-10-2026</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Evaluated tools based on integration with existing development workflows and potential productivity benefits.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38899685036)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -806,6 +806,28 @@
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>16-10-2026</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>1. Worked on the Integration API and investigated existing issues.
+2. Identified and rectified issues affecting API functionality and data processing.
+3. Verified the affected flows to ensure consistent API behavior.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 38904200653)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1356,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1625,6 +1625,28 @@
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>16-10-2026</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued the backend implementation of the Raise Ticket / Support Desk feature, building on the completed frontend integration.
+2. Continued working on backend APIs and database integration for ticket creation, ticket management, and support team assignment.
+3. Continued implementing role-based access control and backend functionality for Service Categories, Support Service Team management, and ticket status updates.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39601388203)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1356,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1647,6 +1647,28 @@
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>21-10-2026</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued the backend implementation of the Raise Ticket / Support Desk feature, building on the completed frontend integration.
+2. Continued working on backend APIs and database integration for ticket creation, ticket management, and support team assignment.
+3. Continued implementing role-based access control and backend functionality for Service Categories, Support Service Team management, and ticket status updates.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39601885062)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1056,7 +1056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1340,6 +1340,27 @@
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>21-10-2026</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued integrating the new storage service into the local application code to enable document uploads through the updated service.
+2. Worked on integrating frontend functionality to access and retrieve files from the new storage service.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39769509097)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1040,6 +1040,26 @@
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>21-10-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>1. Reviewed about the Stored Files Implemented in Last week</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39769644386)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1060,6 +1060,26 @@
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>22-10-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>1. Review about the GIGW Guideliness for the Web portal</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39774264693)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1417,7 +1417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1730,6 +1730,28 @@
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>22-10-2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>"1. Continued the backend implementation of the Raise Ticket / Support Desk feature, building on the completed frontend integration.
+2. Continued working on backend APIs and database integration for ticket creation, ticket management, and support team assignment.
+3. Continued implementing role-based access control and backend functionality for Service Categories, Support Service Team management, and ticket status updates."</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39774434819)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1401,6 +1401,27 @@
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>22-10-2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued integrating the new storage service into the local application code to support document uploads through the updated service.
+2. Worked on integrating backend functionality to access and retrieve files from the new storage service.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39949519992)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1080,6 +1080,26 @@
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>23-10-2026</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>1. Review about the GIGW Guideliness for the Web portal</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39949982378)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1116,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1442,6 +1442,27 @@
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>23-10-2026</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued integrating the new storage service into the local application code to support document uploads through the updated service.
+2. Worked on integrating backend functionality to access and retrieve files from the new storage service.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39950675716)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1479,7 +1479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1814,6 +1814,28 @@
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>23-10-2026</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>1. Continued the backend implementation of the Raise Ticket / Support Desk feature, building on the completed frontend integration.
+2. Continued working on backend APIs and database integration for ticket creation, ticket management, and support team assignment.
+3. Continued implementing role-based access control and backend functionality for Service Categories, Support Service Team management, and ticket status updates.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39957855152)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -828,6 +828,29 @@
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>22-10-2026</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>1. Developed a responsive Password Reset page using React and CSS.
+2. Added current password, new password, and confirm password fields.
+3. Integrated Font Awesome icons for password visibility toggling.
+4. Ensured responsive design for desktop, tablet, and mobile devices.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 39957975341)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -851,6 +851,29 @@
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>23-10-2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>1. Implemented client-side password validation, including required fields, 12–128 character length, and alphanumeric and special character requirements.
+2. Added validation to ensure the new password differs from the current password and matches the confirmation.
+3. Integrated backend API submission with loading states and success/error handling.
+4. Prepared the changes and documentation for pull request review.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40319136258)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1162,7 +1162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1509,6 +1509,28 @@
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>26-10-2026</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>1. Completed the integration of the new storage service into the local application code to support document uploads through the updated service.
+2. Attended a technical talk on “Applying LLMs to Secure Software Development” to gain insights into leveraging large language models for secure software development.
+3. Attended an internal team meeting to discuss the improvements suggested by CDAC Hyderabad and review potential enhancements to the project.</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40325774765)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1547,7 +1547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1904,6 +1904,28 @@
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>26-10-2026</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>1. Attended the “Applying LLMs to Secure Software Development” demo session.
+2. Had discussions with the team and team lead regarding upcoming implementation plans and new features.
+3. Continued implementing backend functionality for role-based access control, Service Categories, Support Service Team management, and ticket status updates.</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40498736857)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -890,7 +890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1146,6 +1146,27 @@
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>26-10-2026</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>1. Review about the GIGW Guideliness for the Web portal
+2. Had a meeting with the web portal team (Regarding Hydrabad visit and discussed the flows)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40499263013)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -890,7 +890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1167,6 +1167,27 @@
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>27-10-2026</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>1. Infrastructure Requirements Review – Reviewed the infrastructure requirements and required hardware specifications for the Web Portal and CDAC Hyderabad – Ongoing 
+2. Server Virtualization and Infrastructure Architecture – Explored server virtualization and reviewed how to design the infrastructure architecture for the Web Portal – Ongoing</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40499534612)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1589,7 +1589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1968,6 +1968,28 @@
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>27-10-2026</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>"1. Continued the backend implementation of the Raise Ticket / Support Desk feature, building on the completed frontend integration.
+2. Continued working on backend APIs and database integration for ticket creation, ticket management, and support team assignment.
+3. Continued implementing role-based access control and backend functionality for Service Categories, Support Service Team management, and ticket status updates."</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40499726389)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1204,7 +1204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1573,6 +1573,26 @@
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>27-10-2026</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>1. Tested the integration of the new storage service into the local application code to support document uploads through the updated service.</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40509526357)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -874,6 +874,27 @@
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>26-10-2026</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>1. Had a meeting with the web portal team (regarding the Hyderabad visit and discussed the flows).
+2. Went through the updated Homepage and checked for possible changes to components.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40509866417)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -895,6 +895,26 @@
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>27-10-2026</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Been a member of the interview panel and conducted interviews for freshers.</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40685000544)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1245,7 +1245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1634,6 +1634,27 @@
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>28-10-2026</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>1. Modified the integration of the new storage service in the local application code to support document uploads through the updated service.
+2. Prepared documentation for client registration based on the new architecture, incorporating the NDA document into the registration workflow.</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40819954533)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1229,6 +1229,26 @@
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>29-10-2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>1. Production Infrastructure Specification and Documentation – Finalized the infrastructure requirements for the Web Portal and CDAC Hyderabad, including CPU, RAM, storage, operating system, and network specifications.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40869043014)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1240,15 +1240,35 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
+          <t>28-10-2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>1. Production Infrastructure Specification and Documentation – Finalized the infrastructure requirements for the Web Portal and CDAC Hyderabad, including CPU, RAM, storage, operating system, and network specifications.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
           <t>29-10-2026</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>1. Production Infrastructure Specification and Documentation – Finalized the infrastructure requirements for the Web Portal and CDAC Hyderabad, including CPU, RAM, storage, operating system, and network specifications.</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40869516659)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -1285,7 +1285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1695,6 +1695,27 @@
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>29-10-2026</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>1. Pushed the new storage service integration code to support document uploads through the updated service.
+2. Prepared documentation for client registration based on the new architecture, incorporating the NDA document into the registration workflow.</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40881821015)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -915,6 +915,27 @@
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>28-10-2026</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>1. Designed the user_access_profiles schema for multiple role–organization mappings.
+2. Defined profile management, primary/secondary profiles, and RBAC validation.</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 40882067171)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -936,6 +936,28 @@
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>29-10-2026</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>1. Designed the pre-authentication and profile-selection flow.
+2. Defined API endpoints and JWT generation after profile validation.
+3. Identified security requirements for token expiry, authorization, and profile switching.</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 41055015671)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -974,7 +974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1312,6 +1312,26 @@
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>30-10-2026</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>1. User &amp; Role Management – Role Matrix and Role Switch Matrix: Reviewed the new role matrix and role-switch matrix, and explored the proposed role-management structure, role permissions, and implementation approach – Ongoing</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Daily status update (run 41064015747)
</commit_message>
<xml_diff>
--- a/daily_status.xlsx
+++ b/daily_status.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -958,6 +958,29 @@
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>30-10-2026</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>1. Refined the database design for managing multiple user profiles across roles and organizations.
+2. Worked on the authentication flow to support profile selection before generating access tokens.
+3. Defined backend validation for authorized role and organization switching.
+4. Reviewed pre-authentication approaches and associated security considerations.</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>